<commit_message>
Mejora del gráfico: eje X multilínea, grillado mensual y ajuste del botón
</commit_message>
<xml_diff>
--- a/data/TSM_is.xlsx
+++ b/data/TSM_is.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\[39]HTML_SIOFEN\Monitoreo\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96326BB0-4EC2-4070-9BF2-BFDFA100D483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{456E22DD-1327-49D6-BD6A-8EEAF38767D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,6 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$W$745</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Hoja2!$I$1:$R$752</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="102">
   <si>
     <t>Idi</t>
   </si>
@@ -354,8 +355,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="166" formatCode="d\.m"/>
-    <numFmt numFmtId="167" formatCode="dd\.mm"/>
+    <numFmt numFmtId="165" formatCode="d\.m"/>
+    <numFmt numFmtId="166" formatCode="dd\.mm"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -517,7 +518,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -551,10 +552,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -565,13 +566,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -631,6 +632,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -70179,14 +70183,14 @@
       <c r="H511" s="6">
         <v>14</v>
       </c>
-      <c r="I511" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="J511" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="K511" s="16" t="s">
-        <v>28</v>
+      <c r="I511" s="46">
+        <v>28.87</v>
+      </c>
+      <c r="J511" s="30">
+        <v>22.33</v>
+      </c>
+      <c r="K511" s="30">
+        <v>21.67</v>
       </c>
       <c r="L511" s="27">
         <v>20.100000000000001</v>
@@ -70200,8 +70204,8 @@
       <c r="O511" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="P511" s="16" t="s">
-        <v>31</v>
+      <c r="P511" s="30">
+        <v>19.97</v>
       </c>
       <c r="Q511" s="27">
         <v>22.6</v>
@@ -70242,8 +70246,8 @@
       <c r="I512" s="2">
         <v>29.3</v>
       </c>
-      <c r="J512" s="16" t="s">
-        <v>33</v>
+      <c r="J512" s="30">
+        <v>22.67</v>
       </c>
       <c r="K512" s="30">
         <v>22.33</v>
@@ -70300,7 +70304,7 @@
         <v>16</v>
       </c>
       <c r="I513" s="2"/>
-      <c r="J513" s="16" t="s">
+      <c r="J513" s="27" t="s">
         <v>39</v>
       </c>
       <c r="K513" s="16" t="s">
@@ -70358,7 +70362,7 @@
         <v>17</v>
       </c>
       <c r="I514" s="2"/>
-      <c r="J514" s="21" t="s">
+      <c r="J514" s="27" t="s">
         <v>44</v>
       </c>
       <c r="K514" s="20"/>
@@ -70377,8 +70381,8 @@
       <c r="P514" s="2">
         <v>20.9</v>
       </c>
-      <c r="Q514" s="21" t="s">
-        <v>40</v>
+      <c r="Q514" s="30">
+        <v>21.17</v>
       </c>
       <c r="R514" s="21" t="s">
         <v>46</v>
@@ -70412,7 +70416,7 @@
       <c r="I515" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J515" s="21" t="s">
+      <c r="J515" s="27" t="s">
         <v>48</v>
       </c>
       <c r="K515" s="21" t="s">
@@ -70472,7 +70476,7 @@
       <c r="I516" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="J516" s="21" t="s">
+      <c r="J516" s="27" t="s">
         <v>33</v>
       </c>
       <c r="K516" s="21" t="s">
@@ -70532,7 +70536,7 @@
       <c r="I517" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="J517" s="21" t="s">
+      <c r="J517" s="27" t="s">
         <v>33</v>
       </c>
       <c r="K517" s="27">
@@ -70592,7 +70596,7 @@
       <c r="I518" s="2">
         <v>28.5</v>
       </c>
-      <c r="J518" s="21" t="s">
+      <c r="J518" s="27" t="s">
         <v>39</v>
       </c>
       <c r="K518" s="21" t="s">
@@ -70652,7 +70656,7 @@
       <c r="I519" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="J519" s="21" t="s">
+      <c r="J519" s="27" t="s">
         <v>66</v>
       </c>
       <c r="K519" s="27">
@@ -70710,7 +70714,7 @@
         <v>23</v>
       </c>
       <c r="I520" s="20"/>
-      <c r="J520" s="21" t="s">
+      <c r="J520" s="27" t="s">
         <v>71</v>
       </c>
       <c r="K520" s="21">
@@ -70768,7 +70772,7 @@
         <v>24</v>
       </c>
       <c r="I521" s="20"/>
-      <c r="J521" s="21" t="s">
+      <c r="J521" s="27" t="s">
         <v>48</v>
       </c>
       <c r="K521" s="20"/>
@@ -70880,7 +70884,7 @@
         <v>26</v>
       </c>
       <c r="I523" s="27"/>
-      <c r="J523" s="21" t="s">
+      <c r="J523" s="27" t="s">
         <v>49</v>
       </c>
       <c r="K523" s="27">
@@ -71000,7 +71004,7 @@
       <c r="I525" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="J525" s="22" t="s">
+      <c r="J525" s="28" t="s">
         <v>81</v>
       </c>
       <c r="K525" s="22" t="s">
@@ -71060,7 +71064,7 @@
       <c r="I526" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="J526" s="22" t="s">
+      <c r="J526" s="28" t="s">
         <v>81</v>
       </c>
       <c r="K526" s="22" t="s">
@@ -71118,7 +71122,7 @@
         <v>30</v>
       </c>
       <c r="I527" s="27"/>
-      <c r="J527" s="22" t="s">
+      <c r="J527" s="28" t="s">
         <v>51</v>
       </c>
       <c r="K527" s="22" t="s">
@@ -71176,7 +71180,7 @@
         <v>31</v>
       </c>
       <c r="I528" s="27"/>
-      <c r="J528" s="22" t="s">
+      <c r="J528" s="28" t="s">
         <v>93</v>
       </c>
       <c r="K528" s="22"/>
@@ -71288,7 +71292,7 @@
       <c r="I530" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="J530" s="21" t="s">
+      <c r="J530" s="27" t="s">
         <v>98</v>
       </c>
       <c r="K530" s="27">
@@ -79178,6 +79182,7 @@
       <c r="O752" s="21"/>
     </row>
   </sheetData>
+  <autoFilter ref="I1:R752" xr:uid="{CC36E404-47A7-476D-A0BA-1C1B7D26C058}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>